<commit_message>
Milestone 3 - Commit 4: Add Lucid CLI Entry
</commit_message>
<xml_diff>
--- a/planner/HGPT_MASTER_PLANNER.xlsx
+++ b/planner/HGPT_MASTER_PLANNER.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MarketingPlan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProjectPlan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MaintenancePlan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QAQCPlan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductionPlan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEOPlan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MarketingPlan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ProjectPlan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MaintenancePlan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="QAQCPlan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ProductionPlan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CEOPlan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>RUNNING</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -519,14 +519,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Lucid</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>MaithuyELEC</t>
@@ -565,14 +562,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Lucid</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>MaithuyELEC</t>

</xml_diff>

<commit_message>
feat(builder): implement BuilderEngine production
</commit_message>
<xml_diff>
--- a/planner/HGPT_MASTER_PLANNER.xlsx
+++ b/planner/HGPT_MASTER_PLANNER.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MarketingPlan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ProjectPlan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MaintenancePlan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="QAQCPlan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ProductionPlan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CEOPlan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MarketingPlan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProjectPlan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MaintenancePlan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QAQCPlan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductionPlan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEOPlan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>GENERATED</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>

<commit_message>
feat(lucid-auto): production workflow v1
</commit_message>
<xml_diff>
--- a/planner/HGPT_MASTER_PLANNER.xlsx
+++ b/planner/HGPT_MASTER_PLANNER.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>GENERATED</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -568,6 +568,49 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>MaithuyELEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AI QAQC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GENERATED</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026/Day013</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Lucid</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>MaithuyELEC</t>
         </is>

</xml_diff>

<commit_message>
Release: Lucid Auto Production v1.0 PASS
</commit_message>
<xml_diff>
--- a/planner/HGPT_MASTER_PLANNER.xlsx
+++ b/planner/HGPT_MASTER_PLANNER.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="180" yWindow="6580" windowWidth="28800" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MarketingPlan" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CEOPlan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -31,7 +30,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -59,7 +60,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -423,7 +424,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="19.6640625" customWidth="1" min="3" max="3"/>
+    <col width="16.83203125" customWidth="1" min="4" max="4"/>
+    <col width="13.33203125" customWidth="1" min="5" max="5"/>
+    <col width="14.33203125" customWidth="1" min="6" max="6"/>
+    <col width="13.6640625" customWidth="1" min="9" max="9"/>
+    <col width="17.5" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -628,7 +637,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -684,7 +693,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -735,7 +744,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -781,7 +790,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -832,7 +841,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(content): unified content pipeline foundation
</commit_message>
<xml_diff>
--- a/planner/HGPT_MASTER_PLANNER.xlsx
+++ b/planner/HGPT_MASTER_PLANNER.xlsx
@@ -596,12 +596,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Facebook,TikTok,Image,Video</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GENERATED</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>